<commit_message>
forward: update frozen E16 E18 E21 real-open ledgers
</commit_message>
<xml_diff>
--- a/forward/e21/E21_forward_dashboard.xlsx
+++ b/forward/e21/E21_forward_dashboard.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signals" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NAV" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fills" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -563,6 +564,67 @@
         <v>0.3074378487744298</v>
       </c>
       <c r="Q2" t="n">
+        <v>0.0338626887492592</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-08-25T09:08:26.098645+00:00</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Crisis</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0.255229225018728</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.0654602418928413</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-0.1897689831258868</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.6586994624763109</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.3074378487744298</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.0338626887492592</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.6586994624763109</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.3074378487744298</v>
+      </c>
+      <c r="Q3" t="n">
         <v>0.0338626887492592</v>
       </c>
     </row>
@@ -577,7 +639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -656,6 +718,37 @@
       </c>
       <c r="I2" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3003385.859672599</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2400122.1596726</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.1324475836892178</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0616352705410217</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0067783498195663</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.799138795950194</v>
+      </c>
+      <c r="H3" t="n">
+        <v>8</v>
+      </c>
+      <c r="I3" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -669,7 +762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -912,6 +1005,600 @@
         <v>103.8</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-25-2880-BUY</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2880</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>2484</v>
+      </c>
+      <c r="F10" t="n">
+        <v>39.8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-25-2886-BUY</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2886</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>2104</v>
+      </c>
+      <c r="F11" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-25-2892-BUY</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2892</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>2925</v>
+      </c>
+      <c r="F12" t="n">
+        <v>33.8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-25-5880-BUY</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>5880</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>3947</v>
+      </c>
+      <c r="F13" t="n">
+        <v>25.05</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-25-2412-BUY</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2412</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>451</v>
+      </c>
+      <c r="F14" t="n">
+        <v>136.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-25-3045-BUY</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>3045</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>533</v>
+      </c>
+      <c r="F15" t="n">
+        <v>115.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-25-4904-BUY</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>4904</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>600</v>
+      </c>
+      <c r="F16" t="n">
+        <v>102.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-25-0050-BUY</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>50</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>195</v>
+      </c>
+      <c r="F17" t="n">
+        <v>104.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>fill_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>signal_date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>fill_date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>side</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>fill_price</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>gross</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>fees_tax</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>slippage_bp</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-24-2880-BUY</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2880</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2517</v>
+      </c>
+      <c r="G2" t="n">
+        <v>39.169575</v>
+      </c>
+      <c r="H2" t="n">
+        <v>98589.82027500001</v>
+      </c>
+      <c r="I2" t="n">
+        <v>84.29429633512498</v>
+      </c>
+      <c r="J2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-24-2886-BUY</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2886</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>2108</v>
+      </c>
+      <c r="G3" t="n">
+        <v>46.873425</v>
+      </c>
+      <c r="H3" t="n">
+        <v>98809.1799</v>
+      </c>
+      <c r="I3" t="n">
+        <v>84.48184881449998</v>
+      </c>
+      <c r="J3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-24-2892-BUY</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2892</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>2945</v>
+      </c>
+      <c r="G4" t="n">
+        <v>33.51674999999999</v>
+      </c>
+      <c r="H4" t="n">
+        <v>98706.82875</v>
+      </c>
+      <c r="I4" t="n">
+        <v>84.39433858124998</v>
+      </c>
+      <c r="J4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-24-5880-BUY</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5880</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>3952</v>
+      </c>
+      <c r="G5" t="n">
+        <v>25.0125</v>
+      </c>
+      <c r="H5" t="n">
+        <v>98849.39999999999</v>
+      </c>
+      <c r="I5" t="n">
+        <v>84.51623699999999</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-24-2412-BUY</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2412</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>450</v>
+      </c>
+      <c r="G6" t="n">
+        <v>136.56825</v>
+      </c>
+      <c r="H6" t="n">
+        <v>61455.7125</v>
+      </c>
+      <c r="I6" t="n">
+        <v>52.5446341875</v>
+      </c>
+      <c r="J6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-24-3045-BUY</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>3045</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>534</v>
+      </c>
+      <c r="G7" t="n">
+        <v>115.0575</v>
+      </c>
+      <c r="H7" t="n">
+        <v>61440.705</v>
+      </c>
+      <c r="I7" t="n">
+        <v>52.531802775</v>
+      </c>
+      <c r="J7" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24-4904-BUY</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4904</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>605</v>
+      </c>
+      <c r="G8" t="n">
+        <v>101.55075</v>
+      </c>
+      <c r="H8" t="n">
+        <v>61438.20374999999</v>
+      </c>
+      <c r="I8" t="n">
+        <v>52.52966420624999</v>
+      </c>
+      <c r="J8" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-24-0050-BUY</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>195</v>
+      </c>
+      <c r="G9" t="n">
+        <v>102.95145</v>
+      </c>
+      <c r="H9" t="n">
+        <v>20075.53275</v>
+      </c>
+      <c r="I9" t="n">
+        <v>17.16458050125</v>
+      </c>
+      <c r="J9" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>